<commit_message>
plain headers, no note row
</commit_message>
<xml_diff>
--- a/results/sep9_meeting/3_similarity_gap_by_model.xlsx
+++ b/results/sep9_meeting/3_similarity_gap_by_model.xlsx
@@ -14,10 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
-  <si>
-    <t xml:space="preserve">Why SapBERT's median sits lower. The 937 correct pairs against the other 720,515. A low median means unrelated pairs are pushed down, which is what leaves room between the two groups.</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t xml:space="preserve">Model</t>
   </si>
@@ -73,9 +70,6 @@
     <t xml:space="preserve">0.05%</t>
   </si>
   <si>
-    <t xml:space="preserve">Median and quartiles for each group, per model.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Group</t>
   </si>
   <si>
@@ -104,9 +98,6 @@
   </si>
   <si>
     <t xml:space="preserve">every other pair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">At each cutoff, correct pairs kept against wrong pairs kept. Cosine step only, before co-occurrence, so these counts are larger than the false positives elsewhere.</t>
   </si>
   <si>
     <t xml:space="preserve">Cosine cutoff</t>
@@ -267,19 +258,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF595959"/>
-      <name val="Calibri"/>
-      <i/>
     </font>
     <font>
       <sz val="11"/>
@@ -308,10 +293,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -619,121 +603,116 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F2" t="n">
+        <v>555</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="n">
+        <v>78236</v>
+      </c>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>9</v>
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.654</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>529</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1675</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B4" t="n">
-        <v>0.916</v>
+        <v>0.704</v>
       </c>
       <c r="C4" t="n">
-        <v>0.841</v>
+        <v>0.161</v>
       </c>
       <c r="D4" t="n">
-        <v>0.075</v>
+        <v>0.543</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9</v>
+        <v>0.75</v>
       </c>
       <c r="F4" t="n">
-        <v>555</v>
+        <v>403</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H4" t="n">
-        <v>78236</v>
+        <v>361</v>
       </c>
       <c r="I4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.654</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.434</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F5" t="n">
-        <v>529</v>
-      </c>
-      <c r="G5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" t="n">
-        <v>1675</v>
-      </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="n">
-        <v>0.704</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.161</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.543</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F6" t="n">
-        <v>403</v>
-      </c>
-      <c r="G6" t="s">
         <v>17</v>
-      </c>
-      <c r="H6" t="n">
-        <v>361</v>
-      </c>
-      <c r="I6" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -760,209 +739,204 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="n">
+        <v>937</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.912</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="n">
+        <v>720515</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>27</v>
+      <c r="I3" t="n">
+        <v>0.837</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C4" t="n">
         <v>937</v>
       </c>
       <c r="D4" t="n">
-        <v>0.625</v>
+        <v>0.106</v>
       </c>
       <c r="E4" t="n">
-        <v>0.874</v>
+        <v>0.483</v>
       </c>
       <c r="F4" t="n">
-        <v>0.916</v>
+        <v>0.654</v>
       </c>
       <c r="G4" t="n">
-        <v>0.96</v>
+        <v>0.839</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.912</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" t="n">
         <v>720515</v>
       </c>
       <c r="D5" t="n">
-        <v>0.505</v>
+        <v>-0.176</v>
       </c>
       <c r="E5" t="n">
-        <v>0.803</v>
+        <v>0.16</v>
       </c>
       <c r="F5" t="n">
-        <v>0.841</v>
+        <v>0.22</v>
       </c>
       <c r="G5" t="n">
-        <v>0.876</v>
+        <v>0.287</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.837</v>
+        <v>0.228</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C6" t="n">
         <v>937</v>
       </c>
       <c r="D6" t="n">
-        <v>0.106</v>
+        <v>-0.007</v>
       </c>
       <c r="E6" t="n">
-        <v>0.483</v>
+        <v>0.539</v>
       </c>
       <c r="F6" t="n">
-        <v>0.654</v>
+        <v>0.704</v>
       </c>
       <c r="G6" t="n">
-        <v>0.839</v>
+        <v>0.867</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>0.66</v>
+        <v>0.694</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C7" t="n">
         <v>720515</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.176</v>
+        <v>-0.179</v>
       </c>
       <c r="E7" t="n">
-        <v>0.16</v>
+        <v>0.091</v>
       </c>
       <c r="F7" t="n">
-        <v>0.22</v>
+        <v>0.161</v>
       </c>
       <c r="G7" t="n">
-        <v>0.287</v>
+        <v>0.244</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0.228</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="n">
-        <v>937</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-0.007</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.539</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.704</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.867</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.694</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" t="n">
-        <v>720515</v>
-      </c>
-      <c r="D9" t="n">
-        <v>-0.179</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.161</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.244</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="n">
         <v>0.176</v>
       </c>
     </row>
@@ -988,858 +962,853 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>937</v>
+      </c>
+      <c r="D2" t="s">
         <v>30</v>
       </c>
+      <c r="E2" t="n">
+        <v>720515</v>
+      </c>
+      <c r="F2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="B3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>937</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="n">
+        <v>720316</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="C4" t="n">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E4" t="n">
-        <v>720515</v>
+        <v>710356</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="C5" t="n">
-        <v>937</v>
+        <v>927</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E5" t="n">
-        <v>720316</v>
+        <v>672758</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="C6" t="n">
-        <v>936</v>
+        <v>891</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
-        <v>710356</v>
+        <v>550864</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="C7" t="n">
-        <v>927</v>
+        <v>792</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E7" t="n">
-        <v>672758</v>
+        <v>314717</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>555</v>
+      </c>
+      <c r="D8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C8" t="n">
-        <v>891</v>
-      </c>
-      <c r="D8" t="s">
-        <v>41</v>
-      </c>
       <c r="E8" t="n">
-        <v>550864</v>
+        <v>78236</v>
       </c>
       <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
         <v>42</v>
-      </c>
-      <c r="G8" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.85</v>
+        <v>0.92</v>
       </c>
       <c r="C9" t="n">
-        <v>792</v>
+        <v>448</v>
       </c>
       <c r="D9" t="s">
         <v>43</v>
       </c>
       <c r="E9" t="n">
-        <v>314717</v>
+        <v>30712</v>
       </c>
       <c r="F9" t="s">
         <v>44</v>
       </c>
       <c r="G9" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="C10" t="n">
-        <v>555</v>
+        <v>286</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="E10" t="n">
-        <v>78236</v>
+        <v>5607</v>
       </c>
       <c r="F10" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="C11" t="n">
-        <v>448</v>
+        <v>193</v>
       </c>
       <c r="D11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E11" t="n">
-        <v>30712</v>
+        <v>1507</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G11" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="C12" t="n">
-        <v>286</v>
+        <v>159</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E12" t="n">
-        <v>5607</v>
+        <v>408</v>
       </c>
       <c r="F12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G12" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="C13" t="n">
-        <v>193</v>
+        <v>110</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E13" t="n">
-        <v>1507</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G13" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>0.98</v>
+        <v>0.5</v>
       </c>
       <c r="C14" t="n">
-        <v>159</v>
+        <v>680</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E14" t="n">
-        <v>408</v>
+        <v>8366</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G14" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B15" t="n">
-        <v>0.99</v>
+        <v>0.6</v>
       </c>
       <c r="C15" t="n">
-        <v>110</v>
+        <v>529</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="E15" t="n">
-        <v>19</v>
+        <v>1675</v>
       </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="C16" t="n">
-        <v>680</v>
+        <v>411</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E16" t="n">
-        <v>8366</v>
+        <v>341</v>
       </c>
       <c r="F16" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="G16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B17" t="n">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="C17" t="n">
-        <v>529</v>
+        <v>343</v>
       </c>
       <c r="D17" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="E17" t="n">
-        <v>1675</v>
+        <v>142</v>
       </c>
       <c r="F17" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B18" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="C18" t="n">
-        <v>411</v>
+        <v>275</v>
       </c>
       <c r="D18" t="s">
         <v>58</v>
       </c>
       <c r="E18" t="n">
-        <v>341</v>
+        <v>49</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="C19" t="n">
-        <v>343</v>
+        <v>221</v>
       </c>
       <c r="D19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E19" t="n">
-        <v>142</v>
+        <v>11</v>
       </c>
       <c r="F19" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="G19" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B20" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="C20" t="n">
-        <v>275</v>
+        <v>178</v>
       </c>
       <c r="D20" t="s">
         <v>61</v>
       </c>
       <c r="E20" t="n">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="F20" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G20" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" t="n">
-        <v>0.85</v>
+        <v>0.92</v>
       </c>
       <c r="C21" t="n">
-        <v>221</v>
+        <v>162</v>
       </c>
       <c r="D21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E21" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F21" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G21" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="C22" t="n">
-        <v>178</v>
+        <v>135</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G22" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="C23" t="n">
-        <v>162</v>
+        <v>120</v>
       </c>
       <c r="D23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F23" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G23" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="C24" t="n">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="E24" t="n">
         <v>2</v>
       </c>
       <c r="F24" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G24" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="C25" t="n">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="D25" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E25" t="n">
         <v>2</v>
       </c>
       <c r="F25" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G25" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B26" t="n">
-        <v>0.98</v>
+        <v>0.5</v>
       </c>
       <c r="C26" t="n">
-        <v>110</v>
+        <v>752</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>11748</v>
       </c>
       <c r="F26" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="G26" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B27" t="n">
-        <v>0.99</v>
+        <v>0.6</v>
       </c>
       <c r="C27" t="n">
-        <v>99</v>
+        <v>626</v>
       </c>
       <c r="D27" t="s">
         <v>68</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3297</v>
       </c>
       <c r="F27" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="G27" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B28" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="C28" t="n">
-        <v>752</v>
+        <v>473</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E28" t="n">
-        <v>11748</v>
+        <v>793</v>
       </c>
       <c r="F28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G28" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C29" t="n">
+        <v>403</v>
+      </c>
+      <c r="D29" t="s">
         <v>16</v>
       </c>
-      <c r="B29" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C29" t="n">
-        <v>626</v>
-      </c>
-      <c r="D29" t="s">
-        <v>71</v>
-      </c>
       <c r="E29" t="n">
-        <v>3297</v>
+        <v>361</v>
       </c>
       <c r="F29" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="G29" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B30" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="C30" t="n">
-        <v>473</v>
+        <v>325</v>
       </c>
       <c r="D30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E30" t="n">
-        <v>793</v>
+        <v>154</v>
       </c>
       <c r="F30" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="G30" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B31" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="C31" t="n">
-        <v>403</v>
+        <v>257</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
       <c r="E31" t="n">
-        <v>361</v>
+        <v>47</v>
       </c>
       <c r="F31" t="s">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="G31" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="C32" t="n">
-        <v>325</v>
+        <v>198</v>
       </c>
       <c r="D32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E32" t="n">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="F32" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="G32" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B33" t="n">
-        <v>0.85</v>
+        <v>0.92</v>
       </c>
       <c r="C33" t="n">
-        <v>257</v>
+        <v>178</v>
       </c>
       <c r="D33" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="E33" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="G33" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B34" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="C34" t="n">
-        <v>198</v>
+        <v>141</v>
       </c>
       <c r="D34" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E34" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G34" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B35" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="C35" t="n">
-        <v>178</v>
+        <v>117</v>
       </c>
       <c r="D35" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F35" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G35" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B36" t="n">
-        <v>0.95</v>
+        <v>0.98</v>
       </c>
       <c r="C36" t="n">
-        <v>141</v>
+        <v>104</v>
       </c>
       <c r="D36" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F36" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G36" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B37" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="C37" t="n">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="D37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E37" t="n">
         <v>2</v>
       </c>
       <c r="F37" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G37" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
-        <v>16</v>
-      </c>
-      <c r="B38" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="C38" t="n">
-        <v>104</v>
-      </c>
-      <c r="D38" t="s">
-        <v>80</v>
-      </c>
-      <c r="E38" t="n">
-        <v>2</v>
-      </c>
-      <c r="F38" t="s">
-        <v>55</v>
-      </c>
-      <c r="G38" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="C39" t="n">
-        <v>96</v>
-      </c>
-      <c r="D39" t="s">
-        <v>81</v>
-      </c>
-      <c r="E39" t="n">
-        <v>2</v>
-      </c>
-      <c r="F39" t="s">
-        <v>55</v>
-      </c>
-      <c r="G39" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>